<commit_message>
Enhance customer rulebook and SQL functions for initials and full name calculations
- Added a new "Initials" field to the customer rulebook JSON, allowing for the calculation of customer initials based on first and last names.
- Updated the formula for calculating "FullName" to format as "FirstName LastName" for consistency across all entries.
- Modified SQL functions to align with the new naming conventions for customer names, ensuring clarity in data retrieval.
- Adjusted seed data to reflect accurate customer names and initials, improving data integrity across the application.

These updates aim to enhance the clarity and usability of customer information within the rulebook framework.
</commit_message>
<xml_diff>
--- a/rulebook-examples/acme-llc/csv/rulebook.xlsx
+++ b/rulebook-examples/acme-llc/csv/rulebook.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBVersions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBCustomizations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__meta__" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -161,7 +162,7 @@
   <commentList>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Identifier for the customers.</t>
+        <t>Identifier for the cusfdsfdstomers.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -174,14 +175,49 @@
         <t>First Name of the customer - used to make the full name</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Last Name of the customer - used to make the full name</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Full name is computed from the first and last name of the customer</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ERB Rulebook</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>The metadata key (e.g. 'tagline', 'motif_palette', 'substrates'). Unique within the table.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Identifier for this metadata entry. Mirrors MetaKey so the row is addressable by Name like every other table.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>How to interpret the value columns: 'string' (use StringValue), 'object' (parse JsonValue as JSON object), 'array' (parse JsonValue as JSON array).</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Plain string value. Populated when ValueType == 'string'; null otherwise.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>JSON-encoded value. Populated when ValueType == 'object' or 'array'; null when ValueType == 'string'.</t>
       </text>
     </comment>
   </commentList>
@@ -477,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -486,6 +522,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,10 +548,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Initials</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>FullName</t>
         </is>
@@ -540,13 +582,17 @@
           <t>Bobby</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3">
+        <f>LEFT($D2, 1) &amp; LEFT($F2, 1)</f>
+        <v/>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Smith</t>
         </is>
       </c>
-      <c r="F2" s="3">
-        <f>$E2 &amp; ", " &amp; $D2</f>
+      <c r="G2" s="3">
+        <f>$D2 &amp; " " &amp; $F2</f>
         <v/>
       </c>
     </row>
@@ -570,13 +616,17 @@
           <t>Jimmy</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3">
+        <f>LEFT($D3, 1) &amp; LEFT($F3, 1)</f>
+        <v/>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Doe</t>
         </is>
       </c>
-      <c r="F3" s="3">
-        <f>$E3 &amp; ", " &amp; $D3</f>
+      <c r="G3" s="3">
+        <f>$D3 &amp; " " &amp; $F3</f>
         <v/>
       </c>
     </row>
@@ -600,13 +650,17 @@
           <t>Mary</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3">
+        <f>LEFT($D4, 1) &amp; LEFT($F4, 1)</f>
+        <v/>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Jones</t>
         </is>
       </c>
-      <c r="F4" s="3">
-        <f>$E4 &amp; ", " &amp; $D4</f>
+      <c r="G4" s="3">
+        <f>$D4 &amp; " " &amp; $F4</f>
         <v/>
       </c>
     </row>
@@ -959,4 +1013,273 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MetaKey</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ValueType</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>StringValue</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>JsonValue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>tagline</t>
+        </is>
+      </c>
+      <c r="B2" s="3">
+        <f>$A2</f>
+        <v/>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>A one-table customer ledger, filed last-name-first.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>motif</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
+        <f>$A3</f>
+        <v/>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>legal-pad</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>motif_palette</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>$A4</f>
+        <v/>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>{"primary": "#a8941f", "accent": "#4a6741", "ink": "#1f1c0a"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>description_rich</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <f>$A5</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ACME, LLC is the **leanest possible rulebook with real wiring** — a single business table (`Customers`) and two calculated fields that re-derive themselves from raw inputs. Unlike its larger cousin ACME Corporation, there are no projects, no roles, no approval workflows: just a client ledger where every customer carries *two* identifiers at once. `Name` is a slug minted from the email address; `FullName` is the same person reformatted last-name-first, courtroom-style. Edit one raw field and both derived labels rewrite themselves in every substrate — Postgres view, Python class, Excel cell, OWL ontology — with zero application code.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>use_cases</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <f>$A6</f>
+        <v/>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>["**Rename a customer.** Change `jane-smith-email-com`'s `FirstName` from `Bobby` to `Robert` and watch `FullName` recompute to `Smith, Robert` on the next read — same row, same id, new label.", "**Update an email address.** Edit `john.doe@email.com` to `j.doe@example.com`; the `Name` slug re-derives to `j.doe-example.com` automatically in every substrate.", "**Add a new customer with just the three raw fields** (`EmailAddress`, `FirstName`, `LastName`) and let the rulebook fill in `Name` and `FullName` — no insert triggers, no application logic.", "**Ask the same question of two substrates.** *\"Sort customers alphabetically by surname.\"* The Postgres view and the Python module both return Doe, Jones, Smith — without anyone writing a sort key.", "**Flip the formula in the rulebook** from `LastName &amp; \", \" &amp; FirstName` to `FirstName &amp; \" \" &amp; LastName` and re-run `effortless build`; every substrate now prints western-style names instead of legal-style, with no migration."]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>signature_rows</t>
+        </is>
+      </c>
+      <c r="B7" s="3">
+        <f>$A7</f>
+        <v/>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>[{"entity": "Customers", "ids": ["jane-smith-email-com", "john-doe-email-com", "emily-jones-email-com"]}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>journal_seed</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <f>$A8</f>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Three customers on file. Each one filed twice — once by email-slug, once by surname-first — and both labels stay in lockstep with the raw fields.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>substrates</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>$A9</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>[{"key": "postgres", "important": true, "chip_label": "Postgres"}, {"key": "excel", "important": true, "chip_label": "Excel"}, {"key": "python", "important": false, "chip_label": "Python"}, {"key": "owl", "important": false, "chip_label": "OWL"}, {"key": "csv", "important": false, "chip_label": "CSV"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>CMCC_Summary</t>
+        </is>
+      </c>
+      <c r="B10" s="3">
+        <f>$A10</f>
+        <v/>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Airtable export with schema-first type mapping: Schemas, Data, Relationships (FK links), Lookups (INDEX/MATCH), Aggregations (SUMIFS/COUNTIFS/Rollups), and Calculated fields (formulas) in Excel dialect. Field types are determined from Airtable's schema metadata FIRST (no coercion); the build FAILS if metadata is unavailable rather than silently inferring from formula/data analysis.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>conversion_metadata</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <f>$A11</f>
+        <v/>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>{"source_base_id": "appWrXPvXbkgQGOxt", "table_count": 3, "tool_version": "2.0.0", "field_type_mapping": "checkbox→boolean, number→number/integer, multipleRecordLinks→relationship, multipleLookupValues→lookup, rollup→aggregation, count→aggregation, formula→calculated", "export_mode": "schema_first_type_mapping", "type_inference": {"enabled": true, "priority": "airtable_metadata (NO COERCION) → formula_analysis → reference_resolution → data_analysis (last-resort inference; build SHOULD FAIL rather than silently use this)", "airtable_type_mapping": "checkbox→boolean, singleLineText→string, multilineText→string, number→number/integer, datetime→datetime, singleSelect→string, email→string, url→string, phoneNumber→string", "data_coercion_hierarchy": "Only invoked when Airtable schema is unavailable (which SHOULD make the build fail). Coercion order: datetime → number → integer → boolean → base64 → json → string", "nullable_support": true, "error_value_handling": "#NUM!, #ERROR!, #N/A, #REF!, #DIV/0!, #VALUE!, #NAME? are treated as NULL"}}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Squash merge dev-finish-reasoning-demo (v2026-06-25)
Adds naive-set-theory and turek-hitchens example rulebooks, German rulespeak
output, ACME OWL individuals/ontology/SHACL, and removes talisman-advanced.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rulebook-examples/acme-llc/csv/rulebook.xlsx
+++ b/rulebook-examples/acme-llc/csv/rulebook.xlsx
@@ -162,17 +162,22 @@
   <commentList>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Identifier for the cusfdsfdstomers.</t>
+        <t>Identifier for the customer.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Thec ustomers email address</t>
+        <t>The customer's email address</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>First Name of the customer - used to make the full name</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Customer initials — the first letter of FirstName followed by the first letter of LastName.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
@@ -1251,7 +1256,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Airtable export with schema-first type mapping: Schemas, Data, Relationships (FK links), Lookups (INDEX/MATCH), Aggregations (SUMIFS/COUNTIFS/Rollups), and Calculated fields (formulas) in Excel dialect. Field types are determined from Airtable's schema metadata FIRST (no coercion); the build FAILS if metadata is unavailable rather than silently inferring from formula/data analysis.</t>
+          <t>Airtable export with schema-first type mapping. This lean rulebook is a single business table (Customers) of raw fields plus Calculated fields (formulas in Excel dialect); it uses no Relationships, Lookups, or Aggregations. Field types are determined from Airtable's schema metadata FIRST (no coercion); the build FAILS if metadata is unavailable rather than silently inferring from formula/data analysis.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1274,7 +1279,7 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>{"source_base_id": "appWrXPvXbkgQGOxt", "table_count": 3, "tool_version": "2.0.0", "field_type_mapping": "checkbox→boolean, number→number/integer, multipleRecordLinks→relationship, multipleLookupValues→lookup, rollup→aggregation, count→aggregation, formula→calculated", "export_mode": "schema_first_type_mapping", "type_inference": {"enabled": true, "priority": "airtable_metadata (NO COERCION) → formula_analysis → reference_resolution → data_analysis (last-resort inference; build SHOULD FAIL rather than silently use this)", "airtable_type_mapping": "checkbox→boolean, singleLineText→string, multilineText→string, number→number/integer, datetime→datetime, singleSelect→string, email→string, url→string, phoneNumber→string", "data_coercion_hierarchy": "Only invoked when Airtable schema is unavailable (which SHOULD make the build fail). Coercion order: datetime → number → integer → boolean → base64 → json → string", "nullable_support": true, "error_value_handling": "#NUM!, #ERROR!, #N/A, #REF!, #DIV/0!, #VALUE!, #NAME? are treated as NULL"}}</t>
+          <t>{"source_base_id": "appWrXPvXbkgQGOxt", "table_count": 4, "tool_version": "2.0.0", "field_type_mapping": "checkbox→boolean, number→number/integer, multipleRecordLinks→relationship, multipleLookupValues→lookup, rollup→aggregation, count→aggregation, formula→calculated", "export_mode": "schema_first_type_mapping", "type_inference": {"enabled": true, "priority": "airtable_metadata (NO COERCION) → formula_analysis → reference_resolution → data_analysis (last-resort inference; build SHOULD FAIL rather than silently use this)", "airtable_type_mapping": "checkbox→boolean, singleLineText→string, multilineText→string, number→number/integer, datetime→datetime, singleSelect→string, email→string, url→string, phoneNumber→string", "data_coercion_hierarchy": "Only invoked when Airtable schema is unavailable (which SHOULD make the build fail). Coercion order: datetime → number → integer → boolean → base64 → json → string", "nullable_support": true, "error_value_handling": "#NUM!, #ERROR!, #N/A, #REF!, #DIV/0!, #VALUE!, #NAME? are treated as NULL"}}</t>
         </is>
       </c>
     </row>

</xml_diff>